<commit_message>
feat: Implementar tipos_contabilidad para niif4
</commit_message>
<xml_diff>
--- a/prototipo_pcr/inputs/insumos.xlsx
+++ b/prototipo_pcr/inputs/insumos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\samuarta\Proyectos\prototipo-pcr\prototipo_pcr\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F34F96C-0947-49A8-9257-9FD5C742CAAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBC72366-6FC7-4304-9C02-9F940D98DB5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="959" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="959" firstSheet="1" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="param_contabilidad" sheetId="6" r:id="rId1"/>
@@ -46,7 +46,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">tasa_cambio!$A$1:$D$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">tipo_seguro!$A$1:$C$1</definedName>
   </definedNames>
-  <calcPr calcId="191028" calcMode="manual"/>
+  <calcPr calcId="191029" calcMode="manual"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -1555,7 +1555,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9966" uniqueCount="460">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10021" uniqueCount="462">
   <si>
     <t>tipo_insumo</t>
   </si>
@@ -2936,6 +2936,12 @@
   <si>
     <t>ifrs4_corporativo</t>
   </si>
+  <si>
+    <t>nuevo_mensual</t>
+  </si>
+  <si>
+    <t>nuevo_mensual_tres_meses</t>
+  </si>
 </sst>
 </file>
 
@@ -3173,7 +3179,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -3247,7 +3253,6 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="5" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="5" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="165" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -22353,7 +22358,7 @@
   <sheetPr codeName="Hoja2">
     <tabColor theme="4"/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="16.1796875" bestFit="1" customWidth="1"/>
@@ -22386,7 +22391,7 @@
     </row>
     <row r="2" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="10" t="s">
-        <v>14</v>
+        <v>458</v>
       </c>
       <c r="B2" s="10" t="s">
         <v>77</v>
@@ -22406,7 +22411,7 @@
     </row>
     <row r="3" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A3" s="10" t="s">
-        <v>14</v>
+        <v>458</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>77</v>
@@ -22426,7 +22431,7 @@
     </row>
     <row r="4" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A4" s="10" t="s">
-        <v>14</v>
+        <v>458</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>67</v>
@@ -22446,19 +22451,19 @@
     </row>
     <row r="5" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A5" s="10" t="s">
-        <v>30</v>
+        <v>459</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="C5" s="10" t="s">
-        <v>77</v>
-      </c>
-      <c r="D5" s="10" t="s">
-        <v>77</v>
+      <c r="C5" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="D5" s="11" t="s">
+        <v>79</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="F5" s="10">
         <v>0</v>
@@ -22466,21 +22471,81 @@
     </row>
     <row r="6" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A6" s="10" t="s">
-        <v>32</v>
+        <v>459</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="C6" s="10" t="s">
-        <v>77</v>
-      </c>
-      <c r="D6" s="10" t="s">
-        <v>77</v>
+      <c r="C6" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>82</v>
       </c>
       <c r="E6" s="10" t="s">
         <v>77</v>
       </c>
       <c r="F6" s="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A7" s="10" t="s">
+        <v>459</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="E7" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="F7" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A8" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="E8" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="F8" s="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A9" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="F9" s="10">
         <v>0</v>
       </c>
     </row>
@@ -55108,31 +55173,30 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3AB633E-9AEE-C044-8F09-ED4F88978E4B}">
   <sheetPr codeName="Hoja6"/>
-  <dimension ref="A1:V25"/>
+  <dimension ref="A1:V28"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="27.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="27.08984375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.36328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.54296875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="22.453125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.6328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.6328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.6328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.6328125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="16.453125" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="27.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.26953125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.36328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.26953125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="23.08984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="17.1796875" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.08984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.54296875" style="1" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="10.1796875" style="3" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="7.81640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.81640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="20.36328125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="8" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="26.6328125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="26.36328125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="23.81640625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="29.6328125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="27.36328125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="19.36328125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="7.7265625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="17.1796875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="20.6328125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="8.1796875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="26.26953125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="26" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="23.7265625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="29.1796875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="26.90625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="19" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:22" s="5" customFormat="1" x14ac:dyDescent="0.35">
@@ -56787,13 +56851,13 @@
       <c r="R24" s="4">
         <v>45641</v>
       </c>
-      <c r="S24" s="64">
+      <c r="S24" s="63">
         <v>49293</v>
       </c>
       <c r="T24" s="4">
         <v>45641</v>
       </c>
-      <c r="U24" s="64">
+      <c r="U24" s="63">
         <v>49293</v>
       </c>
       <c r="V24" s="59">
@@ -56801,12 +56865,284 @@
       </c>
     </row>
     <row r="25" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="D25" s="61"/>
-      <c r="M25" s="3"/>
-      <c r="Q25" s="4"/>
-      <c r="R25" s="4"/>
-      <c r="S25" s="4"/>
-      <c r="T25" s="4"/>
+      <c r="A25" t="s">
+        <v>461</v>
+      </c>
+      <c r="B25" t="s">
+        <v>10</v>
+      </c>
+      <c r="C25" t="s">
+        <v>13</v>
+      </c>
+      <c r="D25">
+        <v>345675387</v>
+      </c>
+      <c r="E25" s="4">
+        <v>45342</v>
+      </c>
+      <c r="F25">
+        <v>2938431543</v>
+      </c>
+      <c r="G25">
+        <f t="shared" ref="G25" si="2">+F25</f>
+        <v>2938431543</v>
+      </c>
+      <c r="H25" t="s">
+        <v>127</v>
+      </c>
+      <c r="I25" t="str">
+        <f t="shared" ref="I25" si="3">+H25</f>
+        <v>HURTO</v>
+      </c>
+      <c r="J25">
+        <v>345675807</v>
+      </c>
+      <c r="K25" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="L25" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="M25" t="s">
+        <v>91</v>
+      </c>
+      <c r="N25" t="s">
+        <v>145</v>
+      </c>
+      <c r="O25" t="s">
+        <v>143</v>
+      </c>
+      <c r="P25" t="s">
+        <v>115</v>
+      </c>
+      <c r="Q25" s="4">
+        <v>45708</v>
+      </c>
+      <c r="R25" s="4">
+        <v>45718</v>
+      </c>
+      <c r="S25" s="4">
+        <v>45721</v>
+      </c>
+      <c r="T25" s="4">
+        <v>45718</v>
+      </c>
+      <c r="U25" s="4">
+        <v>45721</v>
+      </c>
+      <c r="V25" s="59">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="26" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>460</v>
+      </c>
+      <c r="B26" t="s">
+        <v>10</v>
+      </c>
+      <c r="C26" t="s">
+        <v>13</v>
+      </c>
+      <c r="D26">
+        <v>345675387</v>
+      </c>
+      <c r="E26" s="4">
+        <v>45342</v>
+      </c>
+      <c r="F26">
+        <v>2938431544</v>
+      </c>
+      <c r="G26">
+        <f t="shared" ref="G26:G28" si="4">+F26</f>
+        <v>2938431544</v>
+      </c>
+      <c r="H26" t="s">
+        <v>127</v>
+      </c>
+      <c r="I26" t="str">
+        <f t="shared" ref="I26:I28" si="5">+H26</f>
+        <v>HURTO</v>
+      </c>
+      <c r="J26">
+        <v>345675807</v>
+      </c>
+      <c r="K26" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="L26" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="M26" t="s">
+        <v>91</v>
+      </c>
+      <c r="N26" t="s">
+        <v>145</v>
+      </c>
+      <c r="O26" t="s">
+        <v>143</v>
+      </c>
+      <c r="P26" t="s">
+        <v>115</v>
+      </c>
+      <c r="Q26" s="4">
+        <v>45708</v>
+      </c>
+      <c r="R26" s="4">
+        <v>45689</v>
+      </c>
+      <c r="S26" s="4">
+        <v>45717</v>
+      </c>
+      <c r="T26" s="4">
+        <v>45689</v>
+      </c>
+      <c r="U26" s="4">
+        <v>45717</v>
+      </c>
+      <c r="V26" s="59">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="27" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>460</v>
+      </c>
+      <c r="B27" t="s">
+        <v>10</v>
+      </c>
+      <c r="C27" t="s">
+        <v>13</v>
+      </c>
+      <c r="D27">
+        <v>345675387</v>
+      </c>
+      <c r="E27" s="4">
+        <v>45342</v>
+      </c>
+      <c r="F27">
+        <v>2938431545</v>
+      </c>
+      <c r="G27">
+        <f t="shared" si="4"/>
+        <v>2938431545</v>
+      </c>
+      <c r="H27" t="s">
+        <v>127</v>
+      </c>
+      <c r="I27" t="str">
+        <f t="shared" si="5"/>
+        <v>HURTO</v>
+      </c>
+      <c r="J27">
+        <v>345675807</v>
+      </c>
+      <c r="K27" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="L27" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="M27" t="s">
+        <v>91</v>
+      </c>
+      <c r="N27" t="s">
+        <v>145</v>
+      </c>
+      <c r="O27" t="s">
+        <v>143</v>
+      </c>
+      <c r="P27" t="s">
+        <v>115</v>
+      </c>
+      <c r="Q27" s="4">
+        <v>45708</v>
+      </c>
+      <c r="R27" s="4">
+        <v>45710</v>
+      </c>
+      <c r="S27" s="4">
+        <v>45717</v>
+      </c>
+      <c r="T27" s="4">
+        <v>45688</v>
+      </c>
+      <c r="U27" s="4">
+        <v>45717</v>
+      </c>
+      <c r="V27" s="59">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="28" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>460</v>
+      </c>
+      <c r="B28" t="s">
+        <v>10</v>
+      </c>
+      <c r="C28" t="s">
+        <v>13</v>
+      </c>
+      <c r="D28">
+        <v>345675387</v>
+      </c>
+      <c r="E28" s="4">
+        <v>45342</v>
+      </c>
+      <c r="F28">
+        <v>2938431546</v>
+      </c>
+      <c r="G28">
+        <f t="shared" si="4"/>
+        <v>2938431546</v>
+      </c>
+      <c r="H28" t="s">
+        <v>127</v>
+      </c>
+      <c r="I28" t="str">
+        <f t="shared" si="5"/>
+        <v>HURTO</v>
+      </c>
+      <c r="J28">
+        <v>345675807</v>
+      </c>
+      <c r="K28" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="L28" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="M28" t="s">
+        <v>91</v>
+      </c>
+      <c r="N28" t="s">
+        <v>145</v>
+      </c>
+      <c r="O28" t="s">
+        <v>143</v>
+      </c>
+      <c r="P28" t="s">
+        <v>115</v>
+      </c>
+      <c r="Q28" s="4">
+        <v>45641</v>
+      </c>
+      <c r="R28" s="4">
+        <v>45747</v>
+      </c>
+      <c r="S28" s="4">
+        <v>45762</v>
+      </c>
+      <c r="T28" s="4">
+        <v>45688</v>
+      </c>
+      <c r="U28" s="4">
+        <v>45717</v>
+      </c>
+      <c r="V28" s="59">
+        <v>120</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -56931,7 +57267,7 @@
       <c r="D2" t="s">
         <v>444</v>
       </c>
-      <c r="E2" s="62"/>
+      <c r="E2" s="61"/>
       <c r="F2" s="4">
         <v>45674</v>
       </c>
@@ -56998,7 +57334,7 @@
       <c r="D3" t="s">
         <v>444</v>
       </c>
-      <c r="E3" s="62"/>
+      <c r="E3" s="61"/>
       <c r="F3" s="4">
         <v>45674</v>
       </c>
@@ -57065,7 +57401,7 @@
       <c r="D4" t="s">
         <v>444</v>
       </c>
-      <c r="E4" s="63"/>
+      <c r="E4" s="62"/>
       <c r="F4" s="21">
         <v>45674</v>
       </c>
@@ -57132,7 +57468,7 @@
       <c r="D5" t="s">
         <v>444</v>
       </c>
-      <c r="E5" s="62"/>
+      <c r="E5" s="61"/>
       <c r="F5" s="4">
         <v>45674</v>
       </c>
@@ -57199,7 +57535,7 @@
       <c r="D6" t="s">
         <v>444</v>
       </c>
-      <c r="E6" s="62"/>
+      <c r="E6" s="61"/>
       <c r="F6" s="4">
         <v>45674</v>
       </c>
@@ -57266,7 +57602,7 @@
       <c r="D7" t="s">
         <v>444</v>
       </c>
-      <c r="E7" s="62"/>
+      <c r="E7" s="61"/>
       <c r="F7" s="4">
         <v>45674</v>
       </c>
@@ -57333,7 +57669,7 @@
       <c r="D8" t="s">
         <v>444</v>
       </c>
-      <c r="E8" s="62"/>
+      <c r="E8" s="61"/>
       <c r="F8" s="4">
         <v>45674</v>
       </c>
@@ -57400,7 +57736,7 @@
       <c r="D9" t="s">
         <v>444</v>
       </c>
-      <c r="E9" s="62"/>
+      <c r="E9" s="61"/>
       <c r="F9" s="4">
         <v>45674</v>
       </c>
@@ -57467,7 +57803,7 @@
       <c r="D10" t="s">
         <v>444</v>
       </c>
-      <c r="E10" s="62"/>
+      <c r="E10" s="61"/>
       <c r="F10" s="4">
         <v>45674</v>
       </c>
@@ -57534,7 +57870,7 @@
       <c r="D11" t="s">
         <v>444</v>
       </c>
-      <c r="E11" s="62"/>
+      <c r="E11" s="61"/>
       <c r="F11" s="4">
         <v>45674</v>
       </c>
@@ -57601,7 +57937,7 @@
       <c r="D12" t="s">
         <v>444</v>
       </c>
-      <c r="E12" s="62"/>
+      <c r="E12" s="61"/>
       <c r="F12" s="4">
         <v>45674</v>
       </c>
@@ -57668,7 +58004,7 @@
       <c r="D13" t="s">
         <v>444</v>
       </c>
-      <c r="E13" s="62"/>
+      <c r="E13" s="61"/>
       <c r="F13" s="4">
         <v>45674</v>
       </c>
@@ -57735,7 +58071,7 @@
       <c r="D14" t="s">
         <v>444</v>
       </c>
-      <c r="E14" s="62"/>
+      <c r="E14" s="61"/>
       <c r="F14" s="4">
         <v>45674</v>
       </c>
@@ -57802,7 +58138,7 @@
       <c r="D15" t="s">
         <v>444</v>
       </c>
-      <c r="E15" s="62"/>
+      <c r="E15" s="61"/>
       <c r="F15" s="4">
         <v>45674</v>
       </c>
@@ -57869,7 +58205,7 @@
       <c r="D16" t="s">
         <v>444</v>
       </c>
-      <c r="E16" s="62"/>
+      <c r="E16" s="61"/>
       <c r="F16" s="4">
         <v>45674</v>
       </c>
@@ -57936,7 +58272,7 @@
       <c r="D17" t="s">
         <v>444</v>
       </c>
-      <c r="E17" s="63"/>
+      <c r="E17" s="62"/>
       <c r="F17" s="21">
         <v>45674</v>
       </c>
@@ -59455,26 +59791,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7ab8c0d4-f18b-4fef-b649-c77d178c2495">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="65efab6e-20b9-465e-9733-f0c2ab732419" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101003456B0730C78B347BD7589BC061D6E7A" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="eb47ff602caa7ec4c93498109dbc0598">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7ab8c0d4-f18b-4fef-b649-c77d178c2495" xmlns:ns3="65efab6e-20b9-465e-9733-f0c2ab732419" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="15d39866744b831c8a58edb1b96951e3" ns2:_="" ns3:_="">
     <xsd:import namespace="7ab8c0d4-f18b-4fef-b649-c77d178c2495"/>
@@ -59675,26 +59991,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C685BDB-1785-4A39-A308-4CA166889A49}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CE50E33B-922F-4D33-8831-2DF5BA7F11F6}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="7ab8c0d4-f18b-4fef-b649-c77d178c2495"/>
-    <ds:schemaRef ds:uri="65efab6e-20b9-465e-9733-f0c2ab732419"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7ab8c0d4-f18b-4fef-b649-c77d178c2495">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="65efab6e-20b9-465e-9733-f0c2ab732419" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D43FA500-B4BA-4DED-8DE0-EA4A442F0F3F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -59713,6 +60030,25 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C685BDB-1785-4A39-A308-4CA166889A49}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CE50E33B-922F-4D33-8831-2DF5BA7F11F6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="7ab8c0d4-f18b-4fef-b649-c77d178c2495"/>
+    <ds:schemaRef ds:uri="65efab6e-20b9-465e-9733-f0c2ab732419"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{3c0bd4fe-1111-4d13-8e0c-7c33b9eb7581}" enabled="0" method="" siteId="{3c0bd4fe-1111-4d13-8e0c-7c33b9eb7581}" removed="1"/>

</xml_diff>